<commit_message>
Leva 1: norma e sistema, figura 8 do Caso, regras que leem as figuras e pós-entrega sem reclamação
- Caso integrado, figura 8: "A proposta dos dois medidores esperou…" (I07).
- coerencia.py: as regras de PROIBIDO leem também o texto das figuras
  (aria-label do svg, title e text), no teste completo e no --so; a
  extração de texto e as outras conferências não mudam.
- Autoteste: texto das figuras; --so testado pelo main, com regras
  temporárias que sempre casam, que nunca casam e com id desconhecido.
- N25: Produção (linha 8.5.5) e glossário de Conhecimento deixam de pôr a
  reclamação entre as atividades pós-entrega; regra N25 em PROIBIDO.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Caso-Integrado/Caso-Integrado-modelo.xlsx
+++ b/Caso-Integrado/Caso-Integrado-modelo.xlsx
@@ -1917,11 +1917,11 @@
         </c:ser>
         <c:gapWidth val="70"/>
         <c:overlap val="0"/>
-        <c:axId val="86139810"/>
-        <c:axId val="40389438"/>
+        <c:axId val="46253506"/>
+        <c:axId val="31772177"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86139810"/>
+        <c:axId val="46253506"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1953,7 +1953,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40389438"/>
+        <c:crossAx val="31772177"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1961,7 +1961,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40389438"/>
+        <c:axId val="31772177"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2001,7 +2001,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86139810"/>
+        <c:crossAx val="46253506"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>

</xml_diff>